<commit_message>
Improving and restructure code
</commit_message>
<xml_diff>
--- a/ws.xlsx
+++ b/ws.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18730"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10709"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jay\Downloads\FALL2017\Caterpillar Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sujayshah/ExcelParsing/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{24E7DCB3-BC1D-7949-9214-1760236AC180}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="7236" xr2:uid="{8D38DB33-C587-41A5-A534-4499688D29E5}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="14420" xr2:uid="{8D38DB33-C587-41A5-A534-4499688D29E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -483,162 +484,163 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B9854BD-A2A3-4494-AC62-9F60ECB6DEA5}">
   <dimension ref="B1:PB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="423" width="1.77734375" customWidth="1"/>
-    <col min="424" max="424" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="426" max="426" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="428" max="428" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="430" max="430" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="432" max="432" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="434" max="434" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="436" max="436" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="438" max="438" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="440" max="440" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="442" max="442" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="444" max="444" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="446" max="446" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="448" max="448" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="450" max="450" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="452" max="452" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="454" max="454" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="456" max="456" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="458" max="458" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="460" max="460" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="462" max="462" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="464" max="464" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="466" max="466" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="468" max="468" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="470" max="470" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="472" max="472" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="474" max="474" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="476" max="476" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="478" max="478" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="480" max="480" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="482" max="482" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="484" max="484" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="486" max="486" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="488" max="488" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="490" max="490" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="492" max="492" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="494" max="494" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="496" max="496" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="498" max="498" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="500" max="500" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="502" max="502" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="504" max="504" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="506" max="506" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="508" max="508" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="510" max="510" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="512" max="512" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="514" max="514" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="516" max="516" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="518" max="518" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="520" max="520" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="522" max="522" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="524" max="524" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="526" max="526" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="528" max="528" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="530" max="530" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="532" max="532" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="534" max="534" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="536" max="536" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="538" max="538" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="540" max="540" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="542" max="542" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="544" max="544" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="546" max="546" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="548" max="548" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="550" max="550" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="552" max="552" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="554" max="554" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="556" max="556" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="558" max="558" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="560" max="560" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="562" max="562" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="564" max="564" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="566" max="566" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="568" max="568" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="570" max="570" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="572" max="572" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="574" max="574" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="576" max="576" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="578" max="578" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="580" max="580" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="582" max="582" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="584" max="584" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="586" max="586" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="588" max="588" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="590" max="590" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="592" max="592" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="594" max="594" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="596" max="596" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="598" max="598" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="600" max="600" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="602" max="602" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="604" max="604" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="606" max="606" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="608" max="608" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="610" max="610" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="612" max="612" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="614" max="614" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="616" max="616" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="618" max="618" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="620" max="620" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="622" max="622" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="624" max="624" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="626" max="626" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="628" max="628" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="630" max="630" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="632" max="632" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="634" max="634" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="636" max="636" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="638" max="638" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="640" max="640" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="642" max="642" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="644" max="644" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="646" max="646" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="648" max="648" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="650" max="650" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="652" max="652" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="654" max="654" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="656" max="656" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="658" max="658" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="660" max="660" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="662" max="662" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="664" max="664" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="666" max="666" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="668" max="668" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="670" max="670" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="672" max="672" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="674" max="674" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="676" max="676" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="678" max="678" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="680" max="680" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="682" max="682" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="684" max="684" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="686" max="686" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="688" max="688" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="690" max="690" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="692" max="692" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="694" max="694" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="696" max="696" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="698" max="698" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="700" max="700" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="702" max="702" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="704" max="704" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="706" max="706" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="708" max="708" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="710" max="710" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="712" max="712" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="714" max="714" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="716" max="716" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="718" max="718" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="720" max="720" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="722" max="722" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49" customWidth="1"/>
+    <col min="6" max="423" width="1.83203125" customWidth="1"/>
+    <col min="424" max="424" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="426" max="426" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="428" max="428" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="430" max="430" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="432" max="432" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="434" max="434" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="436" max="436" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="438" max="438" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="440" max="440" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="442" max="442" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="444" max="444" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="446" max="446" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="448" max="448" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="450" max="450" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="452" max="452" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="454" max="454" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="456" max="456" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="458" max="458" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="460" max="460" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="462" max="462" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="464" max="464" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="466" max="466" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="468" max="468" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="470" max="470" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="472" max="472" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="474" max="474" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="476" max="476" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="478" max="478" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="480" max="480" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="482" max="482" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="484" max="484" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="486" max="486" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="488" max="488" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="490" max="490" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="492" max="492" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="494" max="494" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="496" max="496" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="498" max="498" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="500" max="500" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="502" max="502" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="504" max="504" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="506" max="506" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="508" max="508" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="510" max="510" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="512" max="512" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="514" max="514" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="516" max="516" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="518" max="518" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="520" max="520" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="522" max="522" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="524" max="524" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="526" max="526" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="528" max="528" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="530" max="530" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="532" max="532" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="534" max="534" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="536" max="536" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="538" max="538" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="540" max="540" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="542" max="542" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="544" max="544" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="546" max="546" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="548" max="548" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="550" max="550" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="552" max="552" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="554" max="554" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="556" max="556" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="558" max="558" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="560" max="560" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="562" max="562" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="564" max="564" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="566" max="566" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="568" max="568" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="570" max="570" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="572" max="572" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="574" max="574" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="576" max="576" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="578" max="578" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="580" max="580" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="582" max="582" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="584" max="584" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="586" max="586" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="588" max="588" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="590" max="590" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="592" max="592" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="594" max="594" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="596" max="596" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="598" max="598" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="600" max="600" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="602" max="602" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="604" max="604" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="606" max="606" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="608" max="608" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="610" max="610" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="612" max="612" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="614" max="614" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="616" max="616" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="618" max="618" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="620" max="620" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="622" max="622" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="624" max="624" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="626" max="626" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="628" max="628" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="630" max="630" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="632" max="632" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="634" max="634" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="636" max="636" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="638" max="638" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="640" max="640" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="642" max="642" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="644" max="644" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="646" max="646" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="648" max="648" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="650" max="650" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="652" max="652" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="654" max="654" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="656" max="656" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="658" max="658" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="660" max="660" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="662" max="662" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="664" max="664" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="666" max="666" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="668" max="668" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="670" max="670" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="672" max="672" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="674" max="674" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="676" max="676" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="678" max="678" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="680" max="680" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="682" max="682" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="684" max="684" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="686" max="686" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="688" max="688" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="690" max="690" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="692" max="692" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="694" max="694" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="696" max="696" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="698" max="698" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="700" max="700" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="702" max="702" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="704" max="704" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="706" max="706" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="708" max="708" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="710" max="710" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="712" max="712" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="714" max="714" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="716" max="716" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="718" max="718" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="720" max="720" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="722" max="722" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:418" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
         <v>10</v>
       </c>
@@ -1783,52 +1785,52 @@
         <v>43830</v>
       </c>
     </row>
-    <row r="2" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B4" s="11" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B8" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B10" s="8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B11" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:418" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:418" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
         <v>9</v>
       </c>

</xml_diff>